<commit_message>
add 2 more var: split nextcloud into 2 var, add seafile
</commit_message>
<xml_diff>
--- a/docs/comp-analogues.xlsx
+++ b/docs/comp-analogues.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35329458-F866-4C7A-8586-D1384C949911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97CE10EE-1EDB-4F7C-8EAD-7696E8EABC58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{808E598B-5B6C-4D1A-8FA0-06D6AB1A0175}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="54">
   <si>
     <t>Название</t>
   </si>
@@ -104,39 +104,24 @@
     <t>Есть, но не очень гибкое: нельзя формульно указать к чему применять</t>
   </si>
   <si>
-    <t>Судя по документации нужно только допилить регистрацию и всё</t>
-  </si>
-  <si>
     <t>Есть AI ассистент для формул</t>
   </si>
   <si>
     <t>Nextcloud Office</t>
   </si>
   <si>
-    <t>Только через Nextcloud, self-hosted регистрации нет</t>
-  </si>
-  <si>
     <t>Как в excel</t>
   </si>
   <si>
-    <t>Нет, связи с табоицами нет</t>
-  </si>
-  <si>
     <t>Нет</t>
   </si>
   <si>
     <t>Есть, как в excel</t>
   </si>
   <si>
-    <t xml:space="preserve">Есть </t>
-  </si>
-  <si>
     <t>Есть, также присутствует связь с таблицами</t>
   </si>
   <si>
-    <t>Нет важных элементов, много допиливать</t>
-  </si>
-  <si>
     <t>Плюсы (фичи)</t>
   </si>
   <si>
@@ -144,13 +129,82 @@
   </si>
   <si>
     <t>Работа с таблицей как с реляционной БД (работа не с ячейками а столбцами)</t>
+  </si>
+  <si>
+    <t>Выводы</t>
+  </si>
+  <si>
+    <t>Судя по документации нужно только допилить регистрацию</t>
+  </si>
+  <si>
+    <t>Нет смысла рассматривать аналоги, где работа с талблицами реализована как работа с БД</t>
+  </si>
+  <si>
+    <t>Есть REST API, OCS, Webdav</t>
+  </si>
+  <si>
+    <t>Работа в таблице как с таблицей а не БД</t>
+  </si>
+  <si>
+    <t>Нужно искать аналогичные сервисы</t>
+  </si>
+  <si>
+    <t>Есть, аналогичный</t>
+  </si>
+  <si>
+    <t>Nextcloud + OnlyOffice</t>
+  </si>
+  <si>
+    <t>Есть, шустрее чем просто в nextcloud office</t>
+  </si>
+  <si>
+    <t>Идентично</t>
+  </si>
+  <si>
+    <t>Таблицы из OnlyOffice</t>
+  </si>
+  <si>
+    <t>Есть External Links - копирование ячеек в одном облаке из одной таблицы в другую</t>
+  </si>
+  <si>
+    <t>Есть - Заполняемые формы, вроде даже нормально выгружаются в таблицу</t>
+  </si>
+  <si>
+    <t>Улучшенная версия Nextcloud Office</t>
+  </si>
+  <si>
+    <t>Есть Nextcloud Forms (нужно доустановить), только ручная выгрузка в .csv</t>
+  </si>
+  <si>
+    <t>Seafile + OnlyOffice</t>
+  </si>
+  <si>
+    <t>Аналогично как выше в Nextcloud + OnlyOffice</t>
+  </si>
+  <si>
+    <t>Есть интерфейс</t>
+  </si>
+  <si>
+    <t>Не все функции есть</t>
+  </si>
+  <si>
+    <t>Блочная структура аналогичная git хранения данных позволяет ещё быстрее обновлять таблицу, редактируемую несколькими пользователями одновременно</t>
+  </si>
+  <si>
+    <t>Улучшенный вариант облака Nextcloud</t>
+  </si>
+  <si>
+    <t>Пока что выглядит как наилучший кандидат</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Из-за блочной структуры при поломке тяжело вытащить данные, </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,8 +220,22 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -198,8 +266,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF975CCB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -207,11 +287,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -219,14 +314,32 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -562,193 +675,290 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F862427C-88CE-482D-B5B2-075D73301028}">
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="8.88671875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.6640625" style="1" customWidth="1"/>
     <col min="4" max="7" width="8.88671875" style="1" customWidth="1"/>
     <col min="8" max="8" width="16.6640625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5546875" style="1" customWidth="1"/>
     <col min="10" max="10" width="17.5546875" style="1" customWidth="1"/>
     <col min="11" max="11" width="25.5546875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="11" style="1" customWidth="1"/>
+    <col min="12" max="12" width="17.44140625" style="1" customWidth="1"/>
     <col min="13" max="13" width="16.5546875" style="1" customWidth="1"/>
     <col min="14" max="14" width="24.44140625" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="1"/>
+    <col min="15" max="15" width="6.6640625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="22.88671875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="7.109375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="28.88671875" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="M1" s="1" t="s">
+      <c r="L1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="145.19999999999999" x14ac:dyDescent="0.3">
+      <c r="O1" s="4"/>
+      <c r="P1" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="103.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="I2" s="2" t="s">
+      <c r="H2" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="L2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="N2" s="3" t="s">
+      <c r="L2" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" ht="92.4" x14ac:dyDescent="0.3">
+      <c r="M2" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" s="4"/>
+      <c r="P2" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="69.599999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="H3" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="J3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="M3" s="2"/>
-      <c r="N3" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="K3" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="M3" s="3"/>
+      <c r="N3" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="O3" s="4"/>
+      <c r="P3" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="85.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="M4" s="11"/>
+      <c r="N4" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="106.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B5" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
final fix: clean appearance
</commit_message>
<xml_diff>
--- a/docs/comp-analogues.xlsx
+++ b/docs/comp-analogues.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97CE10EE-1EDB-4F7C-8EAD-7696E8EABC58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C31512B-FC63-47E8-A1EE-C27E42CA084A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{808E598B-5B6C-4D1A-8FA0-06D6AB1A0175}"/>
   </bookViews>
@@ -197,7 +197,7 @@
     <t>Пока что выглядит как наилучший кандидат</t>
   </si>
   <si>
-    <t xml:space="preserve">Из-за блочной структуры при поломке тяжело вытащить данные, </t>
+    <t>Из-за блочной структуры при поломке тяжело вытащить данные</t>
   </si>
 </sst>
 </file>
@@ -288,17 +288,17 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
+      <top style="thin">
+        <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -306,12 +306,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -320,25 +320,28 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -675,7 +678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F862427C-88CE-482D-B5B2-075D73301028}">
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1" customWidth="1"/>
@@ -696,8 +699,8 @@
     <col min="19" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -744,47 +747,47 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="103.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1">
+    <row r="2" spans="1:16" ht="103.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>14</v>
       </c>
       <c r="J2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="N2" s="9" t="s">
+      <c r="N2" s="8" t="s">
         <v>32</v>
       </c>
       <c r="O2" s="4"/>
@@ -792,45 +795,45 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="69.599999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1">
+    <row r="3" spans="1:16" ht="69.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="L3" s="6" t="s">
         <v>35</v>
       </c>
       <c r="M3" s="3"/>
-      <c r="N3" s="6" t="s">
+      <c r="N3" s="5" t="s">
         <v>49</v>
       </c>
       <c r="O3" s="4"/>
@@ -838,123 +841,96 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="85.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1">
+    <row r="4" spans="1:16" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>40</v>
       </c>
       <c r="H4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="L4" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="M4" s="11"/>
+      <c r="M4" s="10"/>
       <c r="N4" s="7" t="s">
         <v>44</v>
       </c>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
     </row>
-    <row r="5" spans="1:16" ht="106.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1">
+    <row r="5" spans="1:16" ht="105.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>47</v>
       </c>
       <c r="H5" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="K5" s="10" t="s">
+      <c r="K5" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="M5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="N5" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="P5" s="1" t="s">
+      <c r="O5" s="2"/>
+      <c r="P5" s="2" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add comp 2 best var
</commit_message>
<xml_diff>
--- a/docs/comp-analogues.xlsx
+++ b/docs/comp-analogues.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Prog\Labs\OPRPO\mse1h2026-table\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C31512B-FC63-47E8-A1EE-C27E42CA084A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71BDA321-12EB-470B-9364-9D1D63512C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{808E598B-5B6C-4D1A-8FA0-06D6AB1A0175}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{808E598B-5B6C-4D1A-8FA0-06D6AB1A0175}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -31,12 +31,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="57">
   <si>
     <t>Название</t>
   </si>
@@ -198,6 +201,15 @@
   </si>
   <si>
     <t>Из-за блочной структуры при поломке тяжело вытащить данные</t>
+  </si>
+  <si>
+    <t>Nextcloud: написан на php, больше функционал - не является только облачным хранилищем, поддерживает много плагинов</t>
+  </si>
+  <si>
+    <t>Seafile: написан на C/Python - быстрее работает, LDAP на базовом уровне, нет SSO, блочная структура - защита данных и оптимизация скорости работы с ними</t>
+  </si>
+  <si>
+    <t>Заказчику рекомендуется выбрать одно из этих решений. Если объём данных большой и нужна лучшая скорость - seafile, если больший уже реализованный функционал, как плагины, то Nextcloud.</t>
   </si>
 </sst>
 </file>
@@ -306,7 +318,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -343,6 +355,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -678,7 +693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F862427C-88CE-482D-B5B2-075D73301028}">
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1" customWidth="1"/>
@@ -933,7 +948,72 @@
         <v>52</v>
       </c>
     </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A7" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="13"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A8" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="13"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="13"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A9" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13"/>
+      <c r="L9" s="13"/>
+      <c r="M9" s="13"/>
+      <c r="N9" s="13"/>
+      <c r="O9" s="13"/>
+      <c r="P9" s="13"/>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A7:P7"/>
+    <mergeCell ref="A8:P8"/>
+    <mergeCell ref="A9:P9"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>